<commit_message>
Updated the email format
</commit_message>
<xml_diff>
--- a/TestData/Orders.xlsx
+++ b/TestData/Orders.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="33">
   <si>
     <t>Order ID</t>
   </si>
@@ -93,6 +93,24 @@
   </si>
   <si>
     <t>2026-03-26 17:15:22</t>
+  </si>
+  <si>
+    <t>8091149</t>
+  </si>
+  <si>
+    <t>2026-03-26 17:34:40</t>
+  </si>
+  <si>
+    <t>2004341823</t>
+  </si>
+  <si>
+    <t>2026-03-26 17:56:20</t>
+  </si>
+  <si>
+    <t>8091150</t>
+  </si>
+  <si>
+    <t>2026-03-26 17:57:37</t>
   </si>
 </sst>
 </file>
@@ -137,7 +155,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -272,6 +290,39 @@
         <v>26</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="B13" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="C13" t="s" s="0">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s" s="0">
+        <v>29</v>
+      </c>
+      <c r="B14" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C14" t="s" s="0">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="B15" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="C15" t="s" s="0">
+        <v>32</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>